<commit_message>
Fixed errors when parsing extracted data, and already fills QA excel sheet.
</commit_message>
<xml_diff>
--- a/src/pdf_analysis_simplifier/excel-files/analysis_excel_file.xlsx
+++ b/src/pdf_analysis_simplifier/excel-files/analysis_excel_file.xlsx
@@ -18,6 +18,235 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="72">
+  <si>
+    <t xml:space="preserve">QE1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE1 Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE2 Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE3 Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE4 Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE5 Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE6 Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE7 Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE8 Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Score Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The methodology (Constrained Decomposition Grid - CDG) is adequately tailored to the challenges of disassembly tasks, addressing task sequencing and destructive vs. non-destructive methods effectively."
+    "</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The robotic cell setup and components are described conceptually but lack detailed descriptions of individual hardware components, focusing more on algorithms and simulation results."
+    "</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discussions and conclusions are thorough, supported by metrics such as IGD, hypervolume, and epsilon metrics, showcasing the CDG's superiority."
+    "</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The research is primarily simulation-based, which is clearly stated in the methodology and experimental results sections."
+    "</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No mention is made of publicly available implementation or data used in the study."
+    "</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposed solution is explicitly focused on disassembly tasks, addressing disassembly line balancing and destructive/non-destructive operations."
+    "</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparative results with other methods (MOEA/D and NSGAII) are presented to validate findings."
+    "</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The paper provides a moderately updated review of the state of the art in disassembly line balancing, referencing recent advancements in the field."
+    "</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Author</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of manipulators</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manipulator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automated Cell Components</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vision System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use of CAD model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level of Implementation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level of Automation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process Steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Efficiency Considerations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimization of Disassembly Task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Challenges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How to</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Author</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Number of Manipulators</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Manipulator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Automated Cell Components</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Vision System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Use of CAD Model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Level of Implementation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Level of Automation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Process Steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Efficiency Considerations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Optimization of Disassembly Task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Challenges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"How To</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SiQi Lei et al."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not specified; uses general 'robots' at workstations."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not described in detail."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Focuses on robotic workstations and algorithms (CDG implementation)."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not mentioned."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not specified."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulation."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fully automated."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destructive and non-destructive disassembly tasks."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost and time optimization."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task sequencing and resource allocation."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balancing workload, handling destructive/non-destructive decisions, and precedence constraints."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uses CDG with crossover and mutation operators to optimize task sequencing under constraints."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demonstrates CDG's superior convergence and solution quality compared to MOEA/D and NSGAII."</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -91,12 +320,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -292,26 +529,65 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:Y1"/>
+  <dimension ref="A1:EA3"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="98" min="97" style="1" width="4.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="131" min="131" style="1" width="178.72"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
@@ -320,6 +596,222 @@
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+      <c r="CM1" s="1"/>
+      <c r="CN1" s="1"/>
+      <c r="CO1" s="1"/>
+      <c r="CP1" s="1"/>
+      <c r="CQ1" s="1"/>
+      <c r="CR1" s="1"/>
+      <c r="CU1" s="1"/>
+      <c r="CV1" s="1"/>
+      <c r="CW1" s="1"/>
+      <c r="CX1" s="1"/>
+      <c r="CY1" s="1"/>
+      <c r="CZ1" s="1"/>
+      <c r="DA1" s="1"/>
+      <c r="DB1" s="1"/>
+      <c r="DC1" s="1"/>
+      <c r="DD1" s="1"/>
+      <c r="DE1" s="1"/>
+      <c r="DF1" s="1"/>
+      <c r="DG1" s="1"/>
+      <c r="DH1" s="1"/>
+      <c r="DI1" s="1"/>
+      <c r="DJ1" s="1"/>
+      <c r="DK1" s="1"/>
+      <c r="DL1" s="1"/>
+      <c r="DM1" s="1"/>
+      <c r="DN1" s="1"/>
+      <c r="DO1" s="1"/>
+      <c r="DP1" s="1"/>
+      <c r="DQ1" s="1"/>
+      <c r="DR1" s="1"/>
+      <c r="DS1" s="1"/>
+      <c r="DT1" s="1"/>
+      <c r="DU1" s="1"/>
+      <c r="DV1" s="1"/>
+      <c r="DW1" s="1"/>
+      <c r="DX1" s="1"/>
+      <c r="DY1" s="1"/>
+      <c r="DZ1" s="1"/>
+      <c r="EA1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P2" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q2" s="1" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="AX2" s="1"/>
+      <c r="BQ2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P3" s="0" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q3" s="0" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="AX3" s="1"/>
+      <c r="BQ3" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -337,7 +829,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="P1:AV1"/>
+  <dimension ref="A1:IE3"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="10.16"/>
@@ -356,7 +848,54 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="P1" s="1"/>
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
@@ -389,6 +928,321 @@
       <c r="AT1" s="1"/>
       <c r="AU1" s="1"/>
       <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+      <c r="CM1" s="1"/>
+      <c r="CN1" s="1"/>
+      <c r="CO1" s="1"/>
+      <c r="CP1" s="1"/>
+      <c r="CQ1" s="1"/>
+      <c r="CR1" s="1"/>
+      <c r="CS1" s="1"/>
+      <c r="CT1" s="1"/>
+      <c r="CU1" s="1"/>
+      <c r="CV1" s="1"/>
+      <c r="CW1" s="1"/>
+      <c r="CX1" s="1"/>
+      <c r="CY1" s="1"/>
+      <c r="CZ1" s="1"/>
+      <c r="DA1" s="1"/>
+      <c r="DB1" s="1"/>
+      <c r="DC1" s="1"/>
+      <c r="DD1" s="1"/>
+      <c r="DE1" s="1"/>
+      <c r="DF1" s="1"/>
+      <c r="DG1" s="1"/>
+      <c r="DH1" s="1"/>
+      <c r="DI1" s="1"/>
+      <c r="DJ1" s="1"/>
+      <c r="DK1" s="1"/>
+      <c r="DL1" s="1"/>
+      <c r="DM1" s="1"/>
+      <c r="DN1" s="1"/>
+      <c r="DO1" s="1"/>
+      <c r="DP1" s="1"/>
+      <c r="DQ1" s="1"/>
+      <c r="DR1" s="1"/>
+      <c r="DS1" s="1"/>
+      <c r="DT1" s="1"/>
+      <c r="DU1" s="1"/>
+      <c r="DV1" s="1"/>
+      <c r="DW1" s="1"/>
+      <c r="DX1" s="1"/>
+      <c r="DY1" s="1"/>
+      <c r="DZ1" s="1"/>
+      <c r="EA1" s="1"/>
+      <c r="EB1" s="1"/>
+      <c r="EC1" s="1"/>
+      <c r="ED1" s="1"/>
+      <c r="EE1" s="1"/>
+      <c r="EF1" s="1"/>
+      <c r="EG1" s="1"/>
+      <c r="EH1" s="1"/>
+      <c r="EI1" s="1"/>
+      <c r="EJ1" s="1"/>
+      <c r="EK1" s="1"/>
+      <c r="EL1" s="1"/>
+      <c r="EM1" s="1"/>
+      <c r="EN1" s="1"/>
+      <c r="EO1" s="1"/>
+      <c r="EP1" s="1"/>
+      <c r="EQ1" s="1"/>
+      <c r="ER1" s="1"/>
+      <c r="ES1" s="1"/>
+      <c r="ET1" s="1"/>
+      <c r="EU1" s="1"/>
+      <c r="EV1" s="1"/>
+      <c r="EW1" s="1"/>
+      <c r="EX1" s="1"/>
+      <c r="EY1" s="1"/>
+      <c r="EZ1" s="1"/>
+      <c r="FA1" s="1"/>
+      <c r="FB1" s="1"/>
+      <c r="FC1" s="1"/>
+      <c r="FD1" s="1"/>
+      <c r="FE1" s="1"/>
+      <c r="FF1" s="1"/>
+      <c r="FG1" s="1"/>
+      <c r="FH1" s="1"/>
+      <c r="FI1" s="1"/>
+      <c r="FJ1" s="1"/>
+      <c r="FK1" s="1"/>
+      <c r="FL1" s="1"/>
+      <c r="FM1" s="1"/>
+      <c r="FN1" s="1"/>
+      <c r="FO1" s="1"/>
+      <c r="FP1" s="1"/>
+      <c r="FQ1" s="1"/>
+      <c r="FR1" s="1"/>
+      <c r="FS1" s="1"/>
+      <c r="FT1" s="1"/>
+      <c r="FU1" s="1"/>
+      <c r="FV1" s="1"/>
+      <c r="FW1" s="1"/>
+      <c r="FX1" s="1"/>
+      <c r="FY1" s="1"/>
+      <c r="FZ1" s="1"/>
+      <c r="GA1" s="1"/>
+      <c r="GB1" s="1"/>
+      <c r="GC1" s="1"/>
+      <c r="GD1" s="1"/>
+      <c r="GE1" s="1"/>
+      <c r="GF1" s="1"/>
+      <c r="GG1" s="1"/>
+      <c r="GH1" s="1"/>
+      <c r="GI1" s="1"/>
+      <c r="GJ1" s="1"/>
+      <c r="GK1" s="1"/>
+      <c r="GL1" s="1"/>
+      <c r="GM1" s="1"/>
+      <c r="GN1" s="1"/>
+      <c r="GO1" s="1"/>
+      <c r="GP1" s="1"/>
+      <c r="GQ1" s="1"/>
+      <c r="GR1" s="1"/>
+      <c r="GS1" s="1"/>
+      <c r="GT1" s="1"/>
+      <c r="GU1" s="1"/>
+      <c r="GV1" s="1"/>
+      <c r="GW1" s="1"/>
+      <c r="GX1" s="1"/>
+      <c r="GY1" s="1"/>
+      <c r="GZ1" s="1"/>
+      <c r="HA1" s="1"/>
+      <c r="HB1" s="1"/>
+      <c r="HC1" s="1"/>
+      <c r="HD1" s="1"/>
+      <c r="HE1" s="1"/>
+      <c r="HF1" s="1"/>
+      <c r="HG1" s="1"/>
+      <c r="HH1" s="1"/>
+      <c r="HI1" s="1"/>
+      <c r="HJ1" s="1"/>
+      <c r="HK1" s="1"/>
+      <c r="HL1" s="1"/>
+      <c r="HM1" s="1"/>
+      <c r="HN1" s="1"/>
+      <c r="HO1" s="1"/>
+      <c r="HP1" s="1"/>
+      <c r="HQ1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="HR1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="HS1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="HT1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="HU1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="HV1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="HW1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="HX1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="HY1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="HZ1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="IA1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="IB1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="IC1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="ID1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="IE1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="HQ2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="HR2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="HS2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="HT2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="HU2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="HV2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="HW2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="HX2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="HY2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="HZ2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="IA2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="IB2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="IC2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="ID2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="IE2" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="HQ3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="HR3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="HS3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="HT3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="HU3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="HV3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="HW3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="HX3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="HY3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="HZ3" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="IA3" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="IB3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="IC3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="ID3" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="IE3" s="3" t="s">
+        <v>71</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>